<commit_message>
Updated for the new regulator (V3.5)
Signed-off-by: d-el <d2.718l@gmail.com>
</commit_message>
<xml_diff>
--- a/PCB/PS3604LR/output/BOM/Bill of Materials-PS3604LR.xlsx
+++ b/PCB/PS3604LR/output/BOM/Bill of Materials-PS3604LR.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="322">
   <si>
     <t>Designator</t>
   </si>
@@ -60,13 +60,13 @@
     <t>P, N</t>
   </si>
   <si>
-    <t>c375h250</t>
-  </si>
-  <si>
-    <t>PLATED_HOLE2.5_PAD3.75</t>
-  </si>
-  <si>
-    <t>Plated Through Hole: Hole Dia.=2.5mm Pad Dia.=3.75mm</t>
+    <t>c320h180</t>
+  </si>
+  <si>
+    <t>PLATED_HOLE1.8_PAD3.2</t>
+  </si>
+  <si>
+    <t>Plated Through Hole: Hole Dia.=1.8mm Pad Dia.=3.2mm</t>
   </si>
   <si>
     <t>B9, B10, B11</t>
@@ -108,7 +108,7 @@
     <t>CC0805_680PF_50V_5%_NP0</t>
   </si>
   <si>
-    <t>C3, C5, C6, C11, C13, C17, C18, C20, C22, C24, C27, C28, C32, C33, C36, C38, C40, C45, C48, C49, C59, C60, C67, C72, C73</t>
+    <t>C3, C5, C6, C10, C12, C16, C17, C19, C21, C23, C26, C27, C31, C32, C35, C38, C43, C48, C54, C55, C66, C67, C74, C77, C78</t>
   </si>
   <si>
     <t>1u</t>
@@ -129,7 +129,7 @@
     <t>CC0805_330PF_50V_5%_NP0</t>
   </si>
   <si>
-    <t>C7, C16, C23, C25, C26, C30, C31, C35, C39, C41, C46, C47, C50, C51, C52, C55, C58, C61, C62, C63, C68, C69, C70, C71, C74, C75, C76</t>
+    <t>C7, C15, C22, C24, C25, C29, C30, C37, C40, C41, C47, C49, C56, C57, C58, C59, C62, C63, C65, C68, C69, C70, C71, C75, C76, C79, C80</t>
   </si>
   <si>
     <t>100n</t>
@@ -147,7 +147,7 @@
     <t>CC0402_10NF_50V_10%_X7R</t>
   </si>
   <si>
-    <t>C10, C12</t>
+    <t>C11</t>
   </si>
   <si>
     <t>4.7u</t>
@@ -159,7 +159,7 @@
     <t>CC1206_4.7UF_50V_10%_X7R</t>
   </si>
   <si>
-    <t>C14, C15</t>
+    <t>C13, C14</t>
   </si>
   <si>
     <t>2.2u</t>
@@ -168,7 +168,7 @@
     <t>CC1206_2.2UF_100V_10%_X7R</t>
   </si>
   <si>
-    <t>C19, C21</t>
+    <t>C18, C20</t>
   </si>
   <si>
     <t>10u</t>
@@ -177,13 +177,22 @@
     <t>CC1206_10UF_16V_10%_X7R</t>
   </si>
   <si>
-    <t>C29, C66</t>
+    <t>C28, C64</t>
   </si>
   <si>
     <t>CC0402_4.7UF_10V_20%_X5R</t>
   </si>
   <si>
-    <t>C34, C43, C44</t>
+    <t>C33, C36, C42, C46, C50, C51</t>
+  </si>
+  <si>
+    <t>22n</t>
+  </si>
+  <si>
+    <t>CC0402_22NF_16V_10%_X7R</t>
+  </si>
+  <si>
+    <t>C34, C44, C45</t>
   </si>
   <si>
     <t>22u</t>
@@ -195,16 +204,7 @@
     <t>CC1206_22UF_16V_20%_X5R</t>
   </si>
   <si>
-    <t>C37</t>
-  </si>
-  <si>
-    <t>22n</t>
-  </si>
-  <si>
-    <t>CC0402_22NF_16V_10%_X7R</t>
-  </si>
-  <si>
-    <t>C42, C56, C57</t>
+    <t>C39, C60, C61</t>
   </si>
   <si>
     <t>1n</t>
@@ -213,7 +213,7 @@
     <t>CC0402_1NF_50V_5%_NP0</t>
   </si>
   <si>
-    <t>C53, C54</t>
+    <t>C52, C53</t>
   </si>
   <si>
     <t>6.8p</t>
@@ -222,7 +222,7 @@
     <t>CC0402_6.8PF_50V_0.5PF_NP0</t>
   </si>
   <si>
-    <t>C64, C65</t>
+    <t>C72, C73</t>
   </si>
   <si>
     <t>220n</t>
@@ -321,6 +321,18 @@
     <t>Chip Inductors</t>
   </si>
   <si>
+    <t>L3, L4</t>
+  </si>
+  <si>
+    <t>220R@100MHz</t>
+  </si>
+  <si>
+    <t>FB0603_SAMSUNG_CIS10P221NC</t>
+  </si>
+  <si>
+    <t>SMT Ferrite bead</t>
+  </si>
+  <si>
     <t>LD1</t>
   </si>
   <si>
@@ -471,7 +483,7 @@
     <t>General Purpose Thick Film Chip Resistor</t>
   </si>
   <si>
-    <t>R3</t>
+    <t>R3, R35, R38, R45, R47, R51</t>
   </si>
   <si>
     <t>100k</t>
@@ -483,7 +495,7 @@
     <t>R0805_100K_1%_0.125W_100PPM</t>
   </si>
   <si>
-    <t>R4, R8, R25, R55</t>
+    <t>R4, R8, R25, R63</t>
   </si>
   <si>
     <t>1k</t>
@@ -492,7 +504,7 @@
     <t>R0402_1K_1%_0.0625W_100PPM</t>
   </si>
   <si>
-    <t>R5, R6, R29, R30, R31, R32, R47, R49</t>
+    <t>R5, R6, R29, R30, R31, R32, R57, R59</t>
   </si>
   <si>
     <t>100</t>
@@ -513,7 +525,7 @@
     <t>R0603_0R1_1%_0.1W_100PPM</t>
   </si>
   <si>
-    <t>R9, R42</t>
+    <t>R9, R44</t>
   </si>
   <si>
     <t>8k2</t>
@@ -522,7 +534,7 @@
     <t>R0402_8K2_1%_0.0625W_100PPM</t>
   </si>
   <si>
-    <t>R10, R40</t>
+    <t>R10, R43</t>
   </si>
   <si>
     <t>12k</t>
@@ -555,7 +567,7 @@
     <t>R0805_2K2_1%_0.125W_100PPM</t>
   </si>
   <si>
-    <t>R18, R22, R23, R38</t>
+    <t>R18, R22, R23</t>
   </si>
   <si>
     <t>2k</t>
@@ -651,13 +663,31 @@
     <t>R0402_255R_0.1%_0.063W_10PPM</t>
   </si>
   <si>
-    <t>R35</t>
+    <t>R36, R39, R46, R48, R52, R56</t>
+  </si>
+  <si>
+    <t>4k7</t>
+  </si>
+  <si>
+    <t>R0402_4K7_1%_0.0625W_100PPM</t>
+  </si>
+  <si>
+    <t>R37, R42, R61, R62</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>R0402_10K_1%_0.0625W_100PPM</t>
+  </si>
+  <si>
+    <t>R40</t>
   </si>
   <si>
     <t>R0402_12K_0.1%_0.063W_10PPM</t>
   </si>
   <si>
-    <t>R36</t>
+    <t>R41</t>
   </si>
   <si>
     <t>75</t>
@@ -666,31 +696,25 @@
     <t>R0402_75R_0.1%_0.063W_10PPM</t>
   </si>
   <si>
-    <t>R37</t>
-  </si>
-  <si>
-    <t>47k</t>
-  </si>
-  <si>
-    <t>R0603_47K_1%_0.1W_100PPM</t>
-  </si>
-  <si>
-    <t>R39, R41, R51, R52</t>
-  </si>
-  <si>
-    <t>10k</t>
-  </si>
-  <si>
-    <t>R0402_10K_1%_0.0625W_100PPM</t>
-  </si>
-  <si>
-    <t>R43, R44</t>
+    <t>R49, R50</t>
   </si>
   <si>
     <t>R0402_100K_0.1%_0.063W_10PPM</t>
   </si>
   <si>
-    <t>R45, R46</t>
+    <t>R53</t>
+  </si>
+  <si>
+    <t>0R5</t>
+  </si>
+  <si>
+    <t>R0805_0R5_1%_0.125W_200PPM</t>
+  </si>
+  <si>
+    <t>Thin Film Chip Resistor</t>
+  </si>
+  <si>
+    <t>R54, R55</t>
   </si>
   <si>
     <t>8k45</t>
@@ -699,7 +723,7 @@
     <t>R0402_8K45_0.1%_0.063W_10PPM</t>
   </si>
   <si>
-    <t>R48, R50</t>
+    <t>R58, R60</t>
   </si>
   <si>
     <t>0</t>
@@ -711,7 +735,7 @@
     <t>1A (0.05R Max DC Resistance) Zero Ohm Jumper</t>
   </si>
   <si>
-    <t>R53, R54</t>
+    <t>R64, R65</t>
   </si>
   <si>
     <t>13k</t>
@@ -781,7 +805,7 @@
     <t>ESD Protection Diode, Low  Clamping Voltage</t>
   </si>
   <si>
-    <t>U4, U14, U16</t>
+    <t>U4, U15, U16</t>
   </si>
   <si>
     <t>AD8605</t>
@@ -874,7 +898,7 @@
     <t>3 nV/√Hz, Low Power Instrumentation Amplifier</t>
   </si>
   <si>
-    <t>U15</t>
+    <t>U14</t>
   </si>
   <si>
     <t>LMC7101</t>
@@ -919,6 +943,18 @@
     <t>U19</t>
   </si>
   <si>
+    <t>STM32F373CCT6</t>
+  </si>
+  <si>
+    <t>QFP50P900X900X160-48N</t>
+  </si>
+  <si>
+    <t>ARM®Cortex®-M4 32b MCU+FPU, up to 256KB Flash+32KB SRAM, timers, 4 ADCs (16-bit Sig. Delta / 12-bit SAR), 3 DACs, 2 comp., 2.0-3.6 V</t>
+  </si>
+  <si>
+    <t>U20</t>
+  </si>
+  <si>
     <t>AD4680</t>
   </si>
   <si>
@@ -926,18 +962,6 @@
   </si>
   <si>
     <t>Differential Inputs, 1 MSPS/500 kSPS, Dual Simultaneous Sampling SAR ADCs</t>
-  </si>
-  <si>
-    <t>U20</t>
-  </si>
-  <si>
-    <t>STM32F373CCT6</t>
-  </si>
-  <si>
-    <t>QFP50P900X900X160-48N</t>
-  </si>
-  <si>
-    <t>ARM®Cortex®-M4 32b MCU+FPU, up to 256KB Flash+32KB SRAM, timers, 4 ADCs (16-bit Sig. Delta / 12-bit SAR), 3 DACs, 2 comp., 2.0-3.6 V</t>
   </si>
   <si>
     <t>U22</t>
@@ -1328,7 +1352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.796875" customWidth="1"/>
@@ -1556,7 +1580,7 @@
         <v>25</v>
       </c>
       <c r="F11" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
@@ -1627,27 +1651,27 @@
         <v>55</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>25</v>
       </c>
       <c r="F15" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>60</v>
@@ -1656,7 +1680,7 @@
         <v>25</v>
       </c>
       <c r="F16" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
@@ -1867,33 +1891,33 @@
         <v>101</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="F27" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="F28" s="1">
         <v>1</v>
@@ -1913,27 +1937,27 @@
         <v>112</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F29" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="F30" s="1">
         <v>4</v>
@@ -1941,22 +1965,22 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F31" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
@@ -1976,7 +2000,7 @@
         <v>126</v>
       </c>
       <c r="F32" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
@@ -1987,16 +2011,16 @@
         <v>128</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>130</v>
       </c>
       <c r="F33" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
@@ -2007,16 +2031,16 @@
         <v>132</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>134</v>
       </c>
       <c r="F34" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.45">
@@ -2030,10 +2054,10 @@
         <v>137</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="F35" s="1">
         <v>1</v>
@@ -2041,19 +2065,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="F36" s="1">
         <v>1</v>
@@ -2061,42 +2085,42 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="F37" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="F38" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.45">
@@ -2107,56 +2131,56 @@
         <v>155</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F39" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F40" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>163</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F41" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.45">
@@ -2167,33 +2191,33 @@
         <v>165</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F42" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F43" s="1">
         <v>2</v>
@@ -2201,39 +2225,39 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F44" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F45" s="1">
         <v>1</v>
@@ -2241,39 +2265,39 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F46" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>179</v>
+        <v>150</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F47" s="1">
         <v>4</v>
@@ -2281,39 +2305,39 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>155</v>
+        <v>183</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F48" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>184</v>
+        <v>159</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F49" s="1">
         <v>1</v>
@@ -2321,19 +2345,19 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F50" s="1">
         <v>1</v>
@@ -2341,19 +2365,19 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>189</v>
+        <v>162</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F51" s="1">
         <v>1</v>
@@ -2361,19 +2385,19 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>193</v>
+        <v>151</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>194</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
       <c r="F52" s="1">
         <v>1</v>
@@ -2381,19 +2405,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>198</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>149</v>
+        <v>199</v>
       </c>
       <c r="F53" s="1">
         <v>1</v>
@@ -2401,19 +2425,19 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>201</v>
+        <v>151</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>202</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>203</v>
+        <v>153</v>
       </c>
       <c r="F54" s="1">
         <v>1</v>
@@ -2421,19 +2445,19 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>206</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>149</v>
+        <v>207</v>
       </c>
       <c r="F55" s="1">
         <v>1</v>
@@ -2441,19 +2465,19 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F56" s="1">
         <v>1</v>
@@ -2461,19 +2485,19 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>168</v>
+        <v>212</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F57" s="1">
         <v>1</v>
@@ -2481,99 +2505,99 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F58" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F59" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>219</v>
+        <v>172</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F60" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B61" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>147</v>
-      </c>
       <c r="D61" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F61" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>224</v>
+        <v>155</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F62" s="1">
         <v>2</v>
@@ -2581,39 +2605,39 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F63" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F64" s="1">
         <v>2</v>
@@ -2621,13 +2645,13 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>235</v>
+        <v>151</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>236</v>
@@ -2636,10 +2660,10 @@
         <v>237</v>
       </c>
       <c r="F65" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
         <v>238</v>
       </c>
@@ -2647,53 +2671,53 @@
         <v>239</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>242</v>
+      <c r="E66" s="2" t="s">
+        <v>153</v>
       </c>
       <c r="F66" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="D67" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="E67" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="F67" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A68" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="E67" s="2" t="s">
+      <c r="B68" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="F67" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A68" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="D68" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="E68" s="3" t="s">
         <v>250</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>252</v>
       </c>
       <c r="F68" s="1">
         <v>1</v>
@@ -2701,39 +2725,39 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="D69" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="E69" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>247</v>
-      </c>
       <c r="F69" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="C70" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>255</v>
-      </c>
       <c r="D70" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F70" s="1">
         <v>1</v>
@@ -2741,39 +2765,39 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E71" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>262</v>
-      </c>
       <c r="F71" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C72" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="B72" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="D72" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F72" s="1">
         <v>1</v>
@@ -2781,16 +2805,16 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C73" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>269</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>268</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>270</v>
@@ -2807,33 +2831,33 @@
         <v>272</v>
       </c>
       <c r="C74" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="E74" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="E74" s="2" t="s">
-        <v>275</v>
-      </c>
       <c r="F74" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="C75" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="D75" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E75" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>279</v>
       </c>
       <c r="F75" s="1">
         <v>1</v>
@@ -2841,13 +2865,13 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="C76" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>278</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>282</v>
@@ -2867,10 +2891,10 @@
         <v>285</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>255</v>
+        <v>286</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>287</v>
@@ -2887,13 +2911,13 @@
         <v>289</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="E78" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>292</v>
       </c>
       <c r="F78" s="1">
         <v>2</v>
@@ -2901,19 +2925,19 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="C79" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="E79" s="2" t="s">
         <v>295</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>297</v>
       </c>
       <c r="F79" s="1">
         <v>1</v>
@@ -2921,36 +2945,36 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>300</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>299</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F80" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="C81" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="D81" s="2" t="s">
         <v>304</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>303</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>305</v>
@@ -2967,13 +2991,13 @@
         <v>307</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>278</v>
+        <v>308</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>247</v>
+        <v>309</v>
       </c>
       <c r="F82" s="1">
         <v>1</v>
@@ -2981,21 +3005,61 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C83" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>312</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>313</v>
       </c>
       <c r="F83" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A84" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F84" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A85" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F85" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>